<commit_message>
Implement prompt 19 automatic preventive maintenance
</commit_message>
<xml_diff>
--- a/data/excel/planes_preventivos.xlsx
+++ b/data/excel/planes_preventivos.xlsx
@@ -29,6 +29,72 @@
   </x:si>
   <x:si>
     <x:t>ProximaFecha</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FamiliaEquipo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Marca</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Modelo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FrecuenciaHoras</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FrecuenciaKm</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FrecuenciaDias</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ToleranciaHoras</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ToleranciaKm</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ToleranciaDias</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ChecklistCodigo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RepuestosSugeridos</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HHEstimadas</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FechaInicio</x:t>
+  </x:si>
+  <x:si>
+    <x:t>UltimaEjecucionFecha</x:t>
+  </x:si>
+  <x:si>
+    <x:t>UltimaEjecucionHoras</x:t>
+  </x:si>
+  <x:si>
+    <x:t>UltimaEjecucionKm</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ProximaHora</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ProximoKm</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Estado</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Activo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ActualizadoEnUtc</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ActualizadoPor</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -401,10 +467,30 @@
     <x:col min="2" max="2" width="12.853482" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="10.424911" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="8.282054" style="0" customWidth="1"/>
-    <x:col min="5" max="5" width="13.567768" style="0" customWidth="1"/>
+    <x:col min="5" max="6" width="13.567768" style="0" customWidth="1"/>
+    <x:col min="7" max="7" width="6.424911" style="0" customWidth="1"/>
+    <x:col min="8" max="8" width="7.996339" style="0" customWidth="1"/>
+    <x:col min="9" max="9" width="15.710625" style="0" customWidth="1"/>
+    <x:col min="10" max="10" width="13.567768" style="0" customWidth="1"/>
+    <x:col min="11" max="11" width="14.282054" style="0" customWidth="1"/>
+    <x:col min="12" max="12" width="15.282054" style="0" customWidth="1"/>
+    <x:col min="13" max="13" width="13.139196" style="0" customWidth="1"/>
+    <x:col min="14" max="14" width="13.853482" style="0" customWidth="1"/>
+    <x:col min="15" max="15" width="15.139196" style="0" customWidth="1"/>
+    <x:col min="16" max="16" width="19.282054" style="0" customWidth="1"/>
+    <x:col min="17" max="17" width="12.853482" style="0" customWidth="1"/>
+    <x:col min="18" max="18" width="10.853482" style="0" customWidth="1"/>
+    <x:col min="19" max="20" width="20.567768" style="0" customWidth="1"/>
+    <x:col min="21" max="21" width="18.424911" style="0" customWidth="1"/>
+    <x:col min="22" max="22" width="12.710625" style="0" customWidth="1"/>
+    <x:col min="23" max="23" width="11.282054" style="0" customWidth="1"/>
+    <x:col min="24" max="24" width="6.853482" style="0" customWidth="1"/>
+    <x:col min="25" max="25" width="6.282054" style="0" customWidth="1"/>
+    <x:col min="26" max="26" width="16.424911" style="0" customWidth="1"/>
+    <x:col min="27" max="27" width="14.424911" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:5">
+    <x:row r="1" spans="1:27">
       <x:c r="A1" s="1" t="s">
         <x:v>0</x:v>
       </x:c>
@@ -419,6 +505,72 @@
       </x:c>
       <x:c r="E1" s="1" t="s">
         <x:v>4</x:v>
+      </x:c>
+      <x:c r="F1" s="1" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G1" s="1" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H1" s="1" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="I1" s="1" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="J1" s="1" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="K1" s="1" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="L1" s="1" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="M1" s="1" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="N1" s="1" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="O1" s="1" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="P1" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="Q1" s="1" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="R1" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="S1" s="1" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="T1" s="1" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="U1" s="1" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="V1" s="1" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="W1" s="1" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="X1" s="1" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="Y1" s="1" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="Z1" s="1" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="AA1" s="1" t="s">
+        <x:v>26</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>